<commit_message>
style: actualizar la plantilla física de Excel con el total fijo en la fila 34
</commit_message>
<xml_diff>
--- a/storage/ReporteGastosLaborales.xlsx
+++ b/storage/ReporteGastosLaborales.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrador\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrador\MonetarySupport\storage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDD0565F-DD5E-4EDF-A0E2-AD2A3C2B5F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B22C5B-D8F3-41B0-BA7A-3FB6ECD687B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12672" xr2:uid="{6B8A76FC-EF14-4418-8917-5A83E627D679}"/>
+    <workbookView xWindow="3396" yWindow="2460" windowWidth="17280" windowHeight="9060" xr2:uid="{6B8A76FC-EF14-4418-8917-5A83E627D679}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$6:$D$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$6:$D$38</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Gastos Extras no estipulados por facturas, Corredor, Moto Concho y Metro de Santo Domingo, para transportes a Bancas y otros sucesos.</t>
   </si>
@@ -57,54 +57,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>Corredor Ida</t>
-  </si>
-  <si>
-    <t>Metro</t>
-  </si>
-  <si>
-    <t>Entrega equipos Claro TV y Voz</t>
-  </si>
-  <si>
-    <t>Motor</t>
-  </si>
-  <si>
-    <t>P11 Cambiar HDD a SSD Pizarra y Cambio Monitor Perros</t>
-  </si>
-  <si>
-    <t>Metro Ida</t>
-  </si>
-  <si>
-    <t>Uber Moto</t>
-  </si>
-  <si>
-    <t>Revisión PC P40 (verificar SSD/HDD)</t>
-  </si>
-  <si>
-    <t>Uber Regreso</t>
-  </si>
-  <si>
-    <t>Metro Regreso</t>
-  </si>
-  <si>
-    <t>Uber Ida</t>
-  </si>
-  <si>
-    <t>Corredor Regreso</t>
-  </si>
-  <si>
-    <t>P85 Perros - No se veía pantalla exterior</t>
-  </si>
-  <si>
-    <t>P08 Caballos Cambio de HDD a SSD</t>
-  </si>
-  <si>
-    <t>12 Cabecitas RJ45 para reparacion cable video P85</t>
-  </si>
-  <si>
-    <t>Ferreteria al lado de la P85</t>
   </si>
 </sst>
 </file>
@@ -185,7 +137,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -207,9 +159,6 @@
     </xf>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -251,10 +200,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -557,54 +502,54 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.33203125" style="13" customWidth="1"/>
+    <col min="1" max="1" width="40.33203125" style="12" customWidth="1"/>
     <col min="2" max="2" width="25.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="11.5546875" style="1"/>
     <col min="4" max="4" width="17.109375" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
       <c r="E2" s="3"/>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
       <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
       <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -619,351 +564,225 @@
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="4">
-        <v>46167</v>
-      </c>
-      <c r="D7" s="9">
-        <v>50</v>
-      </c>
+      <c r="A7" s="10"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="8"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="4">
-        <v>46167</v>
-      </c>
-      <c r="D8" s="9">
-        <v>20</v>
-      </c>
+      <c r="A8" s="10"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="8"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="4">
-        <v>46167</v>
-      </c>
-      <c r="D9" s="9">
-        <v>20</v>
-      </c>
+      <c r="A9" s="10"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="8"/>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="4">
-        <v>46167</v>
-      </c>
-      <c r="D10" s="9">
-        <v>50</v>
-      </c>
+      <c r="A10" s="10"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="8"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="4">
-        <v>46169</v>
-      </c>
-      <c r="D11" s="9">
-        <v>35</v>
-      </c>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="10"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="8"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="4">
-        <v>46169</v>
-      </c>
-      <c r="D12" s="9">
-        <v>20</v>
-      </c>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="10"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="8"/>
       <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="4">
-        <v>46169</v>
-      </c>
-      <c r="D13" s="9">
-        <v>109.12</v>
-      </c>
+      <c r="A13" s="10"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="8"/>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="4">
-        <v>46169</v>
-      </c>
-      <c r="D14" s="9">
-        <v>20</v>
-      </c>
+      <c r="A14" s="9"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="8"/>
       <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="4">
-        <v>46169</v>
-      </c>
-      <c r="D15" s="9">
-        <v>49.06</v>
-      </c>
+      <c r="A15" s="9"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="8"/>
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="4">
-        <v>46169</v>
-      </c>
-      <c r="D16" s="9">
-        <v>49.02</v>
-      </c>
+      <c r="A16" s="9"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="8"/>
       <c r="E16" s="1"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="4">
-        <v>46169</v>
-      </c>
-      <c r="D17" s="9">
-        <v>20</v>
-      </c>
+      <c r="A17" s="9"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="8"/>
       <c r="E17" s="1"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="4">
-        <v>46169</v>
-      </c>
-      <c r="D18" s="9">
-        <v>35</v>
-      </c>
+      <c r="A18" s="9"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="8"/>
       <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="4">
-        <v>46170</v>
-      </c>
-      <c r="D19" s="9">
-        <v>119.16</v>
-      </c>
+      <c r="A19" s="13"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="8"/>
       <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="4">
-        <v>46170</v>
-      </c>
-      <c r="D20" s="9">
-        <v>149.12</v>
-      </c>
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="8"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="4">
-        <v>46170</v>
-      </c>
-      <c r="D21" s="9">
-        <v>300</v>
-      </c>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="14"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="8"/>
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="1:5" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="10"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="6" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="9"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="9"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="9"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="9"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="9"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="9"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="9"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="9"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="9"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="9"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="9"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="1"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="9"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="1:5" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="A34" s="9"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="7">
-        <f>SUM(D1:D21)</f>
-        <v>1045.48</v>
+      <c r="D34" s="7">
+        <f>SUM(D1:D33)</f>
+        <v>0</v>
       </c>
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="10"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="10"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="1"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="1"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="1"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="10"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="10"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="1"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="10"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="1"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="10"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="1"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="10"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="1"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="10"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="1"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="10"/>
-      <c r="B33" s="5"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="10"/>
-      <c r="B34" s="5"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="9"/>
       <c r="E34" s="1"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="10"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="9"/>
+      <c r="A35" s="11"/>
+      <c r="B35" s="2"/>
       <c r="E35" s="1"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="12"/>
+      <c r="A36" s="11"/>
       <c r="B36" s="2"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="12"/>
+      <c r="A37" s="11"/>
       <c r="B37" s="2"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="12"/>
+      <c r="A38" s="11"/>
       <c r="B38" s="2"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="12"/>
-      <c r="B39" s="2"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A6:D39" xr:uid="{A9BB706F-AAA7-4F18-932C-67237829C53A}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:D39">
-      <sortCondition ref="C6:C39"/>
+  <autoFilter ref="A6:D38" xr:uid="{A9BB706F-AAA7-4F18-932C-67237829C53A}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:D38">
+      <sortCondition ref="C6:C38"/>
     </sortState>
   </autoFilter>
   <mergeCells count="1">

</xml_diff>

<commit_message>
style: subir la versión final de la plantilla ReporteGastosLaborales.xlsx
</commit_message>
<xml_diff>
--- a/storage/ReporteGastosLaborales.xlsx
+++ b/storage/ReporteGastosLaborales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrador\MonetarySupport\storage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B22C5B-D8F3-41B0-BA7A-3FB6ECD687B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B004FBD-E96B-4275-B28D-31E0E7465605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3396" yWindow="2460" windowWidth="17280" windowHeight="9060" xr2:uid="{6B8A76FC-EF14-4418-8917-5A83E627D679}"/>
+    <workbookView xWindow="5544" yWindow="540" windowWidth="17280" windowHeight="9060" xr2:uid="{6B8A76FC-EF14-4418-8917-5A83E627D679}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -757,7 +757,7 @@
         <v>5</v>
       </c>
       <c r="D34" s="7">
-        <f>SUM(D1:D33)</f>
+        <f>SUM(D7:D33)</f>
         <v>0</v>
       </c>
       <c r="E34" s="1"/>

</xml_diff>